<commit_message>
updated example2 comparisons file
</commit_message>
<xml_diff>
--- a/example2-prenormalized/input/comparisons.xlsx
+++ b/example2-prenormalized/input/comparisons.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanmaygandhi/Box Sync/runModac/example2-prenormalized/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD407A11-D709-CD48-8579-9F650ED2B37F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1CCC8BD-4298-794C-8D00-BADDECEE59BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12160" yWindow="5760" windowWidth="14980" windowHeight="15240" xr2:uid="{AC62268A-3574-A143-9B0A-533FA44997D6}"/>
+    <workbookView xWindow="880" yWindow="4160" windowWidth="14980" windowHeight="15240" xr2:uid="{AC62268A-3574-A143-9B0A-533FA44997D6}"/>
   </bookViews>
   <sheets>
     <sheet name="settings" sheetId="6" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="365" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="69">
   <si>
     <t>test</t>
   </si>
@@ -64,9 +64,6 @@
     <t>statistic_selector</t>
   </si>
   <si>
-    <t>p_value</t>
-  </si>
-  <si>
     <t>linear_fc</t>
   </si>
   <si>
@@ -245,6 +242,9 @@
   </si>
   <si>
     <t>method1</t>
+  </si>
+  <si>
+    <t>statistic_cutoff</t>
   </si>
 </sst>
 </file>
@@ -728,7 +728,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{668CCA8B-1A37-364F-8676-16EC9374582A}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17" bestFit="1" customWidth="1"/>
@@ -744,73 +744,65 @@
     </row>
     <row r="2" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="B2">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B3">
-        <v>0.25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>9</v>
+      <c r="A4" s="7" t="s">
+        <v>60</v>
       </c>
       <c r="B4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>61</v>
       </c>
       <c r="B5">
-        <v>41</v>
+        <v>0.25</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="A6" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B6">
-        <v>0.25</v>
+      <c r="B6" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B7" t="s">
         <v>64</v>
       </c>
+      <c r="B7" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="8" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
+      <c r="A8" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="B8" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="B8" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B9" s="7" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>68</v>
-      </c>
-      <c r="B10">
+      <c r="B9">
         <v>25</v>
       </c>
     </row>
@@ -835,7 +827,7 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -851,10 +843,10 @@
         <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D3" s="1"/>
     </row>
@@ -868,314 +860,314 @@
     </row>
     <row r="5" spans="1:4" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
         <v>26</v>
-      </c>
-      <c r="B18" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" t="s">
         <v>39</v>
-      </c>
-      <c r="B30" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B39" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B43" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1200,7 +1192,7 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1216,10 +1208,10 @@
         <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D3" s="1"/>
     </row>
@@ -1233,314 +1225,314 @@
     </row>
     <row r="5" spans="1:4" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
         <v>26</v>
-      </c>
-      <c r="B18" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" t="s">
         <v>39</v>
-      </c>
-      <c r="B30" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B39" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B43" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1564,7 +1556,7 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1580,10 +1572,10 @@
         <v>6</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D3" s="1"/>
     </row>
@@ -1597,314 +1589,314 @@
     </row>
     <row r="5" spans="1:4" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
         <v>26</v>
-      </c>
-      <c r="B18" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" t="s">
         <v>39</v>
-      </c>
-      <c r="B30" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B39" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B43" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1928,7 +1920,7 @@
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1936,30 +1928,30 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1972,314 +1964,314 @@
     </row>
     <row r="5" spans="1:7" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B9" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
         <v>26</v>
-      </c>
-      <c r="B18" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B26" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B29" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" t="s">
         <v>39</v>
-      </c>
-      <c r="B30" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B31" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B35" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B37" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B38" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B39" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B42" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B43" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>